<commit_message>
Team MANTIS: automatic crew routes, street maps, every SLA, rebuilt report and user guides
</commit_message>
<xml_diff>
--- a/ProjectReport/Civic-Operations-Log-Book.xlsx
+++ b/ProjectReport/Civic-Operations-Log-Book.xlsx
@@ -539,7 +539,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NUS ISS, Intelligent Reasoning Systems practice module, Group 23 · 5 September to 20 October 2026</t>
+          <t>NUS ISS, Intelligent Reasoning Systems practice module, Team MANTIS (Group 23) · 5 September to 20 October 2026</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Live on DigitalOcean at http://157.230.191.175/, report and README updated
</commit_message>
<xml_diff>
--- a/ProjectReport/Civic-Operations-Log-Book.xlsx
+++ b/ProjectReport/Civic-Operations-Log-Book.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By member" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log'!$A$1:$E$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log'!$A$1:$E$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -539,7 +539,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NUS ISS, Intelligent Reasoning Systems practice module, Team MANTIS (Group 23) · 5 September to 20 October 2026</t>
+          <t>NUS ISS, Intelligent Reasoning Systems practice module, Team MANTIS (Group 23) · 5 September to 21 October 2026</t>
         </is>
       </c>
     </row>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1895,8 +1895,33 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Nabeel</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Deployment</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Deployed the app on his DigitalOcean server from the public repository, live at http://157.230.191.175/</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Live server, checked 21 Oct</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E47"/>
+  <autoFilter ref="A1:E48"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -2384,7 +2409,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Group report review, corrected experiment cards, live server note
</commit_message>
<xml_diff>
--- a/ProjectReport/Civic-Operations-Log-Book.xlsx
+++ b/ProjectReport/Civic-Operations-Log-Book.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By member" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log'!$A$1:$E$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log'!$A$1:$E$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D11" s="5" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
@@ -708,7 +708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1897,31 +1897,56 @@
     </row>
     <row r="48">
       <c r="A48" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Sankalp</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Crews get their routes automatically with staff pull back, street maps with the depot and the crew's position, a deadline for every request type, linked duplicates that close with their original, group report rebuilt, setup guide and handbook</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>Pull requests 12 and 13 (git, 20 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="n">
         <v>46316</v>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>Nabeel</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Deployed the app on his DigitalOcean server from the public repository, live at http://157.230.191.175/</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>Live server, checked 21 Oct</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E48"/>
+  <autoFilter ref="A1:E49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -2429,7 +2454,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Log book: every dated piece of work and the effort per member
</commit_message>
<xml_diff>
--- a/ProjectReport/Civic-Operations-Log-Book.xlsx
+++ b/ProjectReport/Civic-Operations-Log-Book.xlsx
@@ -11,9 +11,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meetings" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By member" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Effort" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log'!$A$1:$E$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Log'!$A$1:$E$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -539,7 +540,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>NUS ISS, Intelligent Reasoning Systems practice module, Team MANTIS (Group 23) · 5 September to 21 October 2026</t>
+          <t>NUS ISS, Intelligent Reasoning Systems practice module, Team MANTIS (Group 23) · 5 September to 21 October 2026, with the 29 August kickoff</t>
         </is>
       </c>
     </row>
@@ -680,7 +681,7 @@
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>14 MS Teams meetings of over an hour each, from the project start on 5 September. Recorded durations cover 6.5 hours across the meetings in the tracker. See the Meetings sheet.</t>
+          <t>14 MS Teams meetings of over an hour each, from the project start on 5 September. Recorded durations cover 8.5 hours across the meetings in the tracker. See the Meetings sheet.</t>
         </is>
       </c>
     </row>
@@ -708,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -747,7 +748,7 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
-        <v>46270</v>
+        <v>46263</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
@@ -761,7 +762,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: First meeting: system components, evaluation points, dataset, GitHub</t>
+          <t>In person meeting: Kickoff: brainstorming and choosing the project idea</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
@@ -772,7 +773,7 @@
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
@@ -786,7 +787,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Second meeting: report on assigned components, input and output template</t>
+          <t>MS Teams meeting: First meeting: system components, evaluation points, dataset, GitHub</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -797,51 +798,51 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
-        <v>46273</v>
+        <v>46272</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Setup</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>GitHub repository set up: project structure, meeting logs and templates. The full dataset kept local, a documented slice committed</t>
+          <t>MS Teams meeting: Second meeting: report on assigned components, input and output template</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Repository (git, 8 Sep)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
-        <v>46274</v>
+        <v>46273</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Sankalp</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Setup</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Component design and the initial data flow diagram</t>
+          <t>GitHub repository set up: project structure, meeting logs and templates. The full dataset kept local, a documented slice committed</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>Repository (git, 8 Sep)</t>
         </is>
       </c>
     </row>
@@ -851,22 +852,22 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Nabeel</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Design of his two assigned components and the initial data flow diagram, 1.5 hours</t>
+          <t>MS Teams meeting: Component design and the initial data flow diagram</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Tracker (9 Sep)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
@@ -876,47 +877,47 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Nabeel</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Proposal</t>
+          <t>Design</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Proposal kickoff deck, and an architecture that commits to all four technique groups</t>
+          <t>Design of his two assigned components and the initial data flow diagram, 1.5 hours</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>Kickoff deck (git, 9 Sep)</t>
+          <t>Tracker (9 Sep)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
-        <v>46276</v>
+        <v>46274</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Sankalp</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Proposal</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Project proposal content agreed</t>
+          <t>Proposal kickoff deck, and an architecture that commits to all four technique groups</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>Kickoff deck (git, 9 Sep)</t>
         </is>
       </c>
     </row>
@@ -926,47 +927,47 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Nabeel</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>NYC 311 field inventory: complaint families, responsible agencies, the input fields on 311 request pages</t>
+          <t>MS Teams meeting: Project proposal content agreed</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>GitHub (git, 11 Sep)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Nabeel</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Proposal finalised for submission</t>
+          <t>NYC 311 field inventory: complaint families, responsible agencies, the input fields on 311 request pages</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>GitHub (git, 11 Sep)</t>
         </is>
       </c>
     </row>
@@ -976,22 +977,22 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Analysis of the NYC 311 workflow and the mapping from agency to crew skill, 3 hours</t>
+          <t>MS Teams meeting: Proposal finalised for submission</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Tracker (12 Sep)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
@@ -1001,28 +1002,28 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Mohammad</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Proposal</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Project proposal and final system architecture written for submission</t>
+          <t>Analysis of the NYC 311 workflow and the mapping from agency to crew skill, 3 hours</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Proposal (git, 12 Sep), submitted 13 Sep</t>
+          <t>Tracker (12 Sep)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
-        <v>46281</v>
+        <v>46277</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -1031,23 +1032,23 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Proposal</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Post proposal build baseline: data pipeline over NYC 311 Open Data, locked component input and output contracts</t>
+          <t>Project proposal and final system architecture written for submission</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Data pipeline, processed tables, contracts (git, 18 Sep)</t>
+          <t>Proposal (git, 12 Sep), submitted 13 Sep</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>46283</v>
+        <v>46281</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
@@ -1056,17 +1057,17 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Planning</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Planning session: build plan, task board of 31 tasks with owners and due dates, decisions log</t>
+          <t>Post proposal build baseline: data pipeline over NYC 311 Open Data, locked component input and output contracts</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Tracker: Task Board T01 to T31, Decisions Log (tracker)</t>
+          <t>Data pipeline, processed tables, contracts (git, 18 Sep)</t>
         </is>
       </c>
     </row>
@@ -1081,42 +1082,42 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Planning</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Daily demand baselines for Predictive alerting, data preparation notebook rerun</t>
+          <t>Planning session: build plan, task board of 31 tasks with owners and due dates, decisions log</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>Notebook 01 (git, 18 Sep)</t>
+          <t>Tracker: Task Board T01 to T31, Decisions Log (tracker)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
-        <v>46284</v>
+        <v>46283</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Sankalp</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Team meeting</t>
+          <t>Daily demand baselines for Predictive alerting, data preparation notebook rerun</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>Notebook 01 (git, 18 Sep)</t>
         </is>
       </c>
     </row>
@@ -1126,47 +1127,47 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Read Me First guide, a personal reference guide for each member, shared system context for consistent work</t>
+          <t>MS Teams meeting: Team meeting</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>05_Team_Workspace/01_Start_Here and 02_Personal_Guides (git, 19 Sep)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
-        <v>46288</v>
+        <v>46284</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Sankalp</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Team meeting: views for admin, management, crew and citizen, how to show the IRS concepts, core components in the presentation</t>
+          <t>Read Me First guide, a personal reference guide for each member, shared system context for consistent work</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Meeting notes (05_Team_Workspace/08_Meetings, 23 Sep)</t>
+          <t>05_Team_Workspace/01_Start_Here and 02_Personal_Guides (git, 19 Sep)</t>
         </is>
       </c>
     </row>
@@ -1186,18 +1187,18 @@
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Portals and presentation planning</t>
+          <t>Team meeting: views for admin, management, crew and citizen, how to show the IRS concepts, core components in the presentation</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>Meeting notes (05_Team_Workspace/08_Meetings, 23 Sep)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
-        <v>46290</v>
+        <v>46288</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
@@ -1211,7 +1212,7 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Team meeting</t>
+          <t>MS Teams meeting: Portals and presentation planning</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -1226,47 +1227,47 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Khalid</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>First Urgency component upload</t>
+          <t>MS Teams meeting: Team meeting</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t>GitHub upload (git, 25 Sep)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Khalid</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Team meeting</t>
+          <t>First Urgency component upload</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>GitHub upload (git, 25 Sep)</t>
         </is>
       </c>
     </row>
@@ -1276,28 +1277,28 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>Presentation</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Animated demo, research gap table and technique, component and metric tree for the presentation</t>
+          <t>MS Teams meeting: Team meeting</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>04_Course_and_Proposal/03_Proposal_Presentation (git, 26 Sep)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
-        <v>46292</v>
+        <v>46291</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
@@ -1311,22 +1312,22 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Speaker cue card and examiner question preparation</t>
+          <t>Animated demo, research gap table and technique, component and metric tree for the presentation</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Cue card, Examiner Q&amp;A (git, 27 Sep)</t>
+          <t>04_Course_and_Proposal/03_Proposal_Presentation (git, 26 Sep)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="n">
-        <v>46293</v>
+        <v>46292</v>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Sankalp</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -1336,18 +1337,18 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Proposal presentation to the examiners</t>
+          <t>Speaker cue card and examiner question preparation</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Presentation deck, NUS ISS theme (git, 28 Sep)</t>
+          <t>Cue card, Examiner Q&amp;A (git, 27 Sep)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
@@ -1356,23 +1357,23 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Presentation</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Team meeting</t>
+          <t>Proposal presentation to the examiners</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>Presentation deck, NUS ISS theme (git, 28 Sep)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
@@ -1401,22 +1402,22 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Ran the language model experiment notebook on his GPU machine</t>
+          <t>MS Teams meeting: Team meeting</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Verified GPU run results (git, 5 Oct)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1427,7 @@
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Mohammad</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
@@ -1436,18 +1437,18 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Component specification, data findings document, 156 new hand written test lines, second experiment notebook</t>
+          <t>Ran the language model experiment notebook on his GPU machine</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>05_Team_Workspace/03_Specification_and_Contracts (git, 5 Oct)</t>
+          <t>Verified GPU run results (git, 5 Oct)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
@@ -1456,73 +1457,73 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Intake bot, Emergency check, Credibility and Predictive alerting built against the GPU results, evidence pack and experiment register</t>
+          <t>Component specification, data findings document, 156 new hand written test lines, second experiment notebook</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>03_Research/evidence (git, 7 Oct)</t>
+          <t>05_Team_Workspace/03_Specification_and_Contracts (git, 5 Oct)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Nabeel</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Credibility fairness gate closed, glossary, slot filling measured on hand marked spans, contribution report</t>
+          <t>Duplicate detection and Fake request detection v0.1.0: methods, test harness, moved onto the shared component layout</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>Gates in component_status.json (git, 8 Oct)</t>
+          <t>duplicate_detection/docs/CHANGELOG.md (7 Oct)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Sankalp</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Team meeting</t>
+          <t>Intake bot, Emergency check, Credibility and Predictive alerting built against the GPU results, evidence pack and experiment register</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>03_Research/evidence (git, 7 Oct)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
@@ -1531,102 +1532,102 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Shipped models committed, repository tidied</t>
+          <t>Credibility fairness gate closed, glossary, slot filling measured on hand marked spans, contribution report</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t>01_Application/models (git, 9 Oct)</t>
+          <t>Gates in component_status.json (git, 8 Oct)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
-        <v>46306</v>
+        <v>46304</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Khalid</t>
+          <t>All</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>Urgency component: rules, hazard knowledge base, service impact rules, tests</t>
+          <t>MS Teams meeting: Team meeting</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>Branch khalid_code (git, 11 to 13 Oct)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>Sankalp and Khalid</t>
+          <t>Sankalp</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Working session</t>
+          <t>Shipped models committed, repository tidied</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>01_Application/models (git, 9 Oct)</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
-        <v>46310</v>
+        <v>46306</v>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>Khalid</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>Agency and skill routing v1.1.0 with its research report and tests</t>
+          <t>Urgency component: rules, hazard knowledge base, service impact rules, tests</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>Delivered package, report built 15 Oct</t>
+          <t>Branch khalid_code (git, 11 Oct)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="n">
-        <v>46310</v>
+        <v>46307</v>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>Nabeel</t>
+          <t>Khalid</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
@@ -1636,218 +1637,218 @@
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Duplicate detection and Fake request detection, tuned on 295 hand checked real pairs</t>
+          <t>Urgency rules revised, the single file version replaced by the component</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Branch nabeel_c05_c06 (git, 15 Oct)</t>
+          <t>Branch khalid_code (git, 12 Oct)</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Nabeel</t>
+          <t>Khalid</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Research</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Admin questions v1.1.0 benchmarked on 74 gold questions written before any strategy ran, results and change logs</t>
+          <t>Urgency reorganised into its own folder: README, hazard knowledge base, service impact rules, tests. Working session with Sankalp</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>Branch nabeel_c12 (git, 15 Oct)</t>
+          <t>Branch khalid_code (git, 13 Oct), Meetings sheet</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Sankalp and Khalid</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Build</t>
+          <t>Meeting</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>App backend with every component as a measured plugin, citizen, crew and staff portals</t>
+          <t>MS Teams meeting: Working session</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>01_Application/app (git, 15 Oct)</t>
+          <t>Meetings sheet (team record)</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Khalid</t>
+          <t>Mohammad</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>Urgency and Prioritisation final version on his branch</t>
+          <t>Referral advisory rule for Agency and skill routing, learned from the training data</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>Commit 906b77a, pinned in the app (git, 16 Oct)</t>
+          <t>referral_knowledge.json, generated 14 Oct</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Nabeel</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Reviewed Urgency and Prioritisation on a fresh copy, sent findings to Khalid</t>
+          <t>Duplicate pairs labelled by hand on the full real table, matcher tuned, HDBSCAN fix</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>Review message (16 to 18 Oct)</t>
+          <t>duplicate_detection/docs/CHANGELOG.md (14 Oct)</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
-        <v>46313</v>
+        <v>46310</v>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>Khalid</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>External factors v1.0.0 with OpenStreetMap facilities, 90 tests</t>
+          <t>Prioritisation ready for team review: official SLA lookup, starvation protection, ageing, documentation</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>Delivered package (18 Oct)</t>
+          <t>C11_Request_Prioritization/README.md, status dated 15 Oct</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="n">
-        <v>46313</v>
+        <v>46310</v>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Mohammad</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>One folder per component, teammates' components merged, Intake address repair, accounts and roles, Docker containers</t>
+          <t>Agency and skill routing v1.1.0 with its research report and tests. External factors: 4,445 facilities acquired from OpenStreetMap</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>Pull requests 2 and 3 merged (git, 18 Oct)</t>
+          <t>Delivered package, report built 15 Oct. external_factors/data/osm/acquisition_report.json (15 Oct)</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>Nabeel</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Delivery</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>Crew deployment and route optimisation v1.0.0, runtime and full research package</t>
+          <t>Duplicate detection and Fake request detection, tuned on 295 hand checked real pairs</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>GitHub and delivered package (git, 19 Oct)</t>
+          <t>Branch nabeel_c05_c06 (git, 15 Oct)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="n">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>Mohammad</t>
+          <t>Nabeel</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Review</t>
+          <t>Research</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Independent label check of 30 intake test messages</t>
+          <t>Admin questions v1.1.0 benchmarked on 74 gold questions written before any strategy ran, results and change logs</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Returned sheet, 03_Research/experiments (19 Oct)</t>
+          <t>Branch nabeel_c12 (git, 15 Oct)</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
-        <v>46314</v>
+        <v>46310</v>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
@@ -1856,52 +1857,52 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Integration</t>
+          <t>Build</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>Crew deployment plugged in, browser tests at three screen sizes, setup guide, numbered layout, AI ranking reasons on every card</t>
+          <t>App backend with every component as a measured plugin, citizen, crew and staff portals</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>Pull requests 4 and 5 merged (git, 19 Oct)</t>
+          <t>01_Application/app (git, 15 Oct)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Khalid</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Meeting</t>
+          <t>Delivery</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>MS Teams meeting: Team meeting</t>
+          <t>Urgency and Prioritisation final version on his branch</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Meetings sheet (team record)</t>
+          <t>Commit 906b77a, pinned in the app (git, 16 Oct)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n">
-        <v>46315</v>
+        <v>46311</v>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Sankalp</t>
+          <t>Mohammad</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -1911,42 +1912,267 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>Crews get their routes automatically with staff pull back, street maps with the depot and the crew's position, a deadline for every request type, linked duplicates that close with their original, group report rebuilt, setup guide and handbook</t>
+          <t>NYC road network built for crew routing</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
-          <t>Pull requests 12 and 13 (git, 20 Oct)</t>
+          <t>crew_deployment_and_routing roads_manifest.json, built 16 Oct</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Sankalp</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Reviewed Urgency and Prioritisation on a fresh copy, sent findings to Khalid</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Review message (16 to 18 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>Road graph acquired and checked for the route planner</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>crew_deployment_and_routing SOURCE_README.md (17 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>External factors v1.0.0 with OpenStreetMap facilities, 90 tests</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Delivered package (18 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Sankalp</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>One folder per component, teammates' components merged, Intake address repair, accounts and roles, Docker containers</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>Pull requests 2 and 3 merged (git, 18 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="9" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Crew deployment and route optimisation v1.0.0, runtime and full research package</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>GitHub and delivered package (git, 19 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Mohammad</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Independent label check of 30 intake test messages</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>Returned sheet, 03_Research/experiments (19 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="9" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Sankalp</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Integration</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Crew deployment plugged in, browser tests at three screen sizes, setup guide, numbered layout, AI ranking reasons on every card</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Pull requests 4 and 5 merged (git, 19 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Meeting</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>MS Teams meeting: Team meeting</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>Meetings sheet (team record)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Sankalp</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Crews get their routes automatically with staff pull back, street maps with the depot and the crew's position, a deadline for every request type, linked duplicates that close with their original, group report rebuilt, setup guide and handbook</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Pull requests 12 and 13 (git, 20 Oct)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n">
         <v>46316</v>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
         <is>
           <t>Nabeel</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>Deployment</t>
         </is>
       </c>
-      <c r="D49" s="5" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Deployed the app on his DigitalOcean server from the public repository, live at http://157.230.191.175/</t>
         </is>
       </c>
-      <c r="E49" s="5" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>Live server, checked 21 Oct</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E49"/>
+  <autoFilter ref="A1:E58"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1958,7 +2184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1997,16 +2223,16 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
-        <v>46270</v>
+        <v>46263</v>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>MS Teams</t>
+          <t>In person</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>First meeting: system components, evaluation points, dataset, GitHub</t>
+          <t>Kickoff: brainstorming and choosing the project idea</t>
         </is>
       </c>
       <c r="D2" s="4" t="n">
@@ -2020,7 +2246,7 @@
     </row>
     <row r="3">
       <c r="A3" s="9" t="n">
-        <v>46272</v>
+        <v>46270</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
@@ -2029,11 +2255,11 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Second meeting: report on assigned components, input and output template</t>
+          <t>First meeting: system components, evaluation points, dataset, GitHub</t>
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
@@ -2043,7 +2269,7 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
-        <v>46274</v>
+        <v>46272</v>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
@@ -2052,7 +2278,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Component design and the initial data flow diagram</t>
+          <t>Second meeting: report on assigned components, input and output template</t>
         </is>
       </c>
       <c r="D4" s="4" t="n">
@@ -2066,7 +2292,7 @@
     </row>
     <row r="5">
       <c r="A5" s="9" t="n">
-        <v>46276</v>
+        <v>46274</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
@@ -2075,7 +2301,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Project proposal content agreed</t>
+          <t>Component design and the initial data flow diagram</t>
         </is>
       </c>
       <c r="D5" s="5" t="n">
@@ -2089,7 +2315,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
-        <v>46277</v>
+        <v>46276</v>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
@@ -2098,13 +2324,11 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Proposal finalised for submission</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>over 1</t>
-        </is>
+          <t>Project proposal content agreed</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>1.5</v>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
@@ -2114,7 +2338,7 @@
     </row>
     <row r="7">
       <c r="A7" s="9" t="n">
-        <v>46284</v>
+        <v>46277</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
@@ -2123,7 +2347,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Team meeting</t>
+          <t>Proposal finalised for submission</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -2139,7 +2363,7 @@
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
-        <v>46288</v>
+        <v>46284</v>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
@@ -2148,7 +2372,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Portals and presentation planning</t>
+          <t>Team meeting</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2164,7 +2388,7 @@
     </row>
     <row r="9">
       <c r="A9" s="9" t="n">
-        <v>46290</v>
+        <v>46288</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -2173,7 +2397,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Team meeting</t>
+          <t>Portals and presentation planning</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -2189,7 +2413,7 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>46291</v>
+        <v>46290</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
@@ -2214,7 +2438,7 @@
     </row>
     <row r="11">
       <c r="A11" s="9" t="n">
-        <v>46297</v>
+        <v>46291</v>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
@@ -2239,7 +2463,7 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
@@ -2264,7 +2488,7 @@
     </row>
     <row r="13">
       <c r="A13" s="9" t="n">
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
@@ -2289,7 +2513,7 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
@@ -2298,7 +2522,7 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Working session</t>
+          <t>Team meeting</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -2308,37 +2532,62 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Sankalp and Khalid</t>
+          <t>All four members</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>MS Teams</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Working session</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>over 1</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Sankalp and Khalid</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n">
         <v>46315</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>MS Teams</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>Team meeting</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>over 1</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>All four members</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>14 MS Teams meetings in total over the project, each over one hour.</t>
         </is>
@@ -2394,7 +2643,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
@@ -2414,11 +2663,11 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>15 Oct: Agency and skill routing v1.1.0 with its research report and tests. 18 Oct: External factors v1.0.0 with OpenStreetMap facilities, 90 tests. 19 Oct: Crew deployment and route optimisation v1.0.0, runtime and full research package</t>
+          <t>15 Oct: Agency and skill routing v1.1.0 with its research report and tests. External factors: 4,445 facilities acquired from OpenStreetMap. 18 Oct: External factors v1.0.0 with OpenStreetMap facilities, 90 tests. 19 Oct: Crew deployment and route optimisation v1.0.0, runtime and full research package</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
@@ -2434,7 +2683,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -2454,7 +2703,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -2471,4 +2720,168 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Days with dated work</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Meeting hours</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Man-days (lower bound)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Share of the 10 expected</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Khalid Alhazmi</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>93%</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Mohammad Alharthi</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>112%</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Nabeel Taresh</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>82%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Indish Sankalp Sandeep</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>20.3</v>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>203%</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>123% of 40</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>The practice module expects about 10 man-days of effort from each participant, 40 for a team of four. A date with dated work counts as one man-day and meeting hours are added at 8 hours a day. Work without a dated record is not counted, so every figure here is a lower bound.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A8:E8"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Docker build fetches the Intake address tagger from the release page
</commit_message>
<xml_diff>
--- a/ProjectReport/Civic-Operations-Log-Book.xlsx
+++ b/ProjectReport/Civic-Operations-Log-Book.xlsx
@@ -1462,7 +1462,7 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Component specification, data findings document, 156 new hand written test lines, second experiment notebook</t>
+          <t>Component specification, data findings document, 156 new hand written test lines, second experiment ipynb</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Man-days (lower bound)</t>
+          <t>Man days (lower bound)</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
@@ -2873,7 +2873,7 @@
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>The practice module expects about 10 man-days of effort from each participant, 40 for a team of four. A date with dated work counts as one man-day and meeting hours are added at 8 hours a day. Work without a dated record is not counted, so every figure here is a lower bound.</t>
+          <t>The practice module expects about 10 man days of effort from each participant, 40 for a team of four. A date with dated work counts as one man day and meeting hours are added at 8 hours a day. Work without a dated record is not counted, so every figure here is a lower bound.</t>
         </is>
       </c>
     </row>

</xml_diff>